<commit_message>
Inclui novo time na Liga Clássica
</commit_message>
<xml_diff>
--- a/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Completa.xlsx
+++ b/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Completa.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="58">
   <si>
     <t>Rodada 1</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>Rolo Compressor ZN</t>
+  </si>
+  <si>
+    <t>RS Expressões da Arte</t>
   </si>
   <si>
     <t>S.E.R. GRILLO</t>
@@ -550,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1201,16 +1204,16 @@
         <v>41</v>
       </c>
       <c r="B39">
-        <v>84.85986328125</v>
+        <v>58.25</v>
       </c>
       <c r="C39">
-        <v>79.4501953125</v>
+        <v>63.780029296875</v>
       </c>
       <c r="D39">
-        <v>78.93994140625</v>
+        <v>68.43994140625</v>
       </c>
       <c r="E39">
-        <v>78.93994140625</v>
+        <v>68.43994140625</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -1218,16 +1221,16 @@
         <v>42</v>
       </c>
       <c r="B40">
-        <v>60.159912109375</v>
+        <v>84.85986328125</v>
       </c>
       <c r="C40">
-        <v>64.580078125</v>
+        <v>79.4501953125</v>
       </c>
       <c r="D40">
-        <v>88.759765625</v>
+        <v>78.93994140625</v>
       </c>
       <c r="E40">
-        <v>88.759765625</v>
+        <v>78.93994140625</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -1235,16 +1238,16 @@
         <v>43</v>
       </c>
       <c r="B41">
-        <v>49</v>
+        <v>60.159912109375</v>
       </c>
       <c r="C41">
-        <v>36.429931640625</v>
+        <v>64.580078125</v>
       </c>
       <c r="D41">
-        <v>54.35009765625</v>
+        <v>88.759765625</v>
       </c>
       <c r="E41">
-        <v>54.35009765625</v>
+        <v>88.759765625</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -1252,16 +1255,16 @@
         <v>44</v>
       </c>
       <c r="B42">
-        <v>61.659912109375</v>
+        <v>49</v>
       </c>
       <c r="C42">
-        <v>69.5</v>
+        <v>36.429931640625</v>
       </c>
       <c r="D42">
-        <v>83.64990234375</v>
+        <v>54.35009765625</v>
       </c>
       <c r="E42">
-        <v>83.64990234375</v>
+        <v>54.35009765625</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -1269,16 +1272,16 @@
         <v>45</v>
       </c>
       <c r="B43">
-        <v>42.9599609375</v>
+        <v>61.659912109375</v>
       </c>
       <c r="C43">
-        <v>91.47998046875</v>
+        <v>69.5</v>
       </c>
       <c r="D43">
-        <v>99.35986328125</v>
+        <v>83.64990234375</v>
       </c>
       <c r="E43">
-        <v>99.35986328125</v>
+        <v>83.64990234375</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -1286,16 +1289,16 @@
         <v>46</v>
       </c>
       <c r="B44">
-        <v>54.10009765625</v>
+        <v>42.9599609375</v>
       </c>
       <c r="C44">
-        <v>71.5</v>
+        <v>91.47998046875</v>
       </c>
       <c r="D44">
-        <v>67.39990234375</v>
+        <v>99.35986328125</v>
       </c>
       <c r="E44">
-        <v>67.39990234375</v>
+        <v>99.35986328125</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -1303,16 +1306,16 @@
         <v>47</v>
       </c>
       <c r="B45">
-        <v>61.9599609375</v>
+        <v>54.10009765625</v>
       </c>
       <c r="C45">
-        <v>84.47998046875</v>
+        <v>71.5</v>
       </c>
       <c r="D45">
-        <v>87.39990234375</v>
+        <v>67.39990234375</v>
       </c>
       <c r="E45">
-        <v>87.39990234375</v>
+        <v>67.39990234375</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -1320,16 +1323,16 @@
         <v>48</v>
       </c>
       <c r="B46">
-        <v>64.2001953125</v>
+        <v>61.9599609375</v>
       </c>
       <c r="C46">
-        <v>95.3798828125</v>
+        <v>84.47998046875</v>
       </c>
       <c r="D46">
-        <v>56.9599609375</v>
+        <v>87.39990234375</v>
       </c>
       <c r="E46">
-        <v>56.9599609375</v>
+        <v>87.39990234375</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -1337,16 +1340,16 @@
         <v>49</v>
       </c>
       <c r="B47">
-        <v>66.85986328125</v>
+        <v>64.2001953125</v>
       </c>
       <c r="C47">
-        <v>92.7001953125</v>
+        <v>95.3798828125</v>
       </c>
       <c r="D47">
-        <v>72.740234375</v>
+        <v>56.9599609375</v>
       </c>
       <c r="E47">
-        <v>72.740234375</v>
+        <v>56.9599609375</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -1354,16 +1357,16 @@
         <v>50</v>
       </c>
       <c r="B48">
-        <v>58.9599609375</v>
+        <v>66.85986328125</v>
       </c>
       <c r="C48">
-        <v>79.27978515625</v>
+        <v>92.7001953125</v>
       </c>
       <c r="D48">
-        <v>86.66015625</v>
+        <v>72.740234375</v>
       </c>
       <c r="E48">
-        <v>86.66015625</v>
+        <v>72.740234375</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -1371,16 +1374,16 @@
         <v>51</v>
       </c>
       <c r="B49">
-        <v>70</v>
+        <v>58.9599609375</v>
       </c>
       <c r="C49">
-        <v>87.5</v>
+        <v>79.27978515625</v>
       </c>
       <c r="D49">
-        <v>88.06005859375</v>
+        <v>86.66015625</v>
       </c>
       <c r="E49">
-        <v>88.06005859375</v>
+        <v>86.66015625</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -1388,16 +1391,16 @@
         <v>52</v>
       </c>
       <c r="B50">
-        <v>68.06005859375</v>
+        <v>70</v>
       </c>
       <c r="C50">
-        <v>82.18017578125</v>
+        <v>87.5</v>
       </c>
       <c r="D50">
-        <v>105.759765625</v>
+        <v>88.06005859375</v>
       </c>
       <c r="E50">
-        <v>105.759765625</v>
+        <v>88.06005859375</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -1405,16 +1408,16 @@
         <v>53</v>
       </c>
       <c r="B51">
-        <v>51.260009765625</v>
+        <v>68.06005859375</v>
       </c>
       <c r="C51">
-        <v>95.5</v>
+        <v>82.18017578125</v>
       </c>
       <c r="D51">
-        <v>61.159912109375</v>
+        <v>105.759765625</v>
       </c>
       <c r="E51">
-        <v>61.159912109375</v>
+        <v>105.759765625</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -1422,16 +1425,16 @@
         <v>54</v>
       </c>
       <c r="B52">
-        <v>72.16015625</v>
+        <v>51.260009765625</v>
       </c>
       <c r="C52">
-        <v>93.47998046875</v>
+        <v>95.5</v>
       </c>
       <c r="D52">
-        <v>85.259765625</v>
+        <v>61.159912109375</v>
       </c>
       <c r="E52">
-        <v>85.259765625</v>
+        <v>61.159912109375</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -1439,16 +1442,16 @@
         <v>55</v>
       </c>
       <c r="B53">
-        <v>55.89990234375</v>
+        <v>72.16015625</v>
       </c>
       <c r="C53">
-        <v>77.3798828125</v>
+        <v>93.47998046875</v>
       </c>
       <c r="D53">
-        <v>43.909912109375</v>
+        <v>85.259765625</v>
       </c>
       <c r="E53">
-        <v>43.909912109375</v>
+        <v>85.259765625</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -1456,15 +1459,32 @@
         <v>56</v>
       </c>
       <c r="B54">
-        <v>0</v>
+        <v>55.89990234375</v>
       </c>
       <c r="C54">
-        <v>0</v>
+        <v>77.3798828125</v>
       </c>
       <c r="D54">
-        <v>0</v>
+        <v>43.909912109375</v>
       </c>
       <c r="E54">
+        <v>43.909912109375</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55">
+        <v>0</v>
+      </c>
+      <c r="C55">
+        <v>0</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
         <v>0</v>
       </c>
     </row>
@@ -1475,7 +1495,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:A54"/>
+  <dimension ref="A2:A55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="1:1">
@@ -1741,6 +1761,11 @@
     <row r="54" spans="1:1">
       <c r="A54" s="1" t="s">
         <v>56</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" s="1" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1750,7 +1775,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1768,7 +1793,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1776,7 +1801,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1784,7 +1809,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1792,7 +1817,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1800,7 +1825,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1808,7 +1833,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1816,7 +1841,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1824,7 +1849,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1832,7 +1857,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1840,7 +1865,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1848,7 +1873,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1856,7 +1881,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -1864,7 +1889,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1872,7 +1897,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -1880,7 +1905,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1888,7 +1913,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1896,7 +1921,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -1904,7 +1929,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -1912,7 +1937,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -1920,7 +1945,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -1928,7 +1953,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -1936,7 +1961,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -1944,7 +1969,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -1952,7 +1977,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -1960,7 +1985,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -1976,7 +2001,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -1984,7 +2009,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -2072,7 +2097,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -2080,7 +2105,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -2168,9 +2193,17 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="B53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54">
         <v>0</v>
       </c>
     </row>
@@ -2181,7 +2214,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2191,7 +2224,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2">
         <v>84.85986328125</v>
@@ -2247,7 +2280,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B9">
         <v>72.16015625</v>
@@ -2263,7 +2296,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B11">
         <v>70</v>
@@ -2271,7 +2304,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B12">
         <v>68.06005859375</v>
@@ -2287,7 +2320,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B14">
         <v>66.85986328125</v>
@@ -2319,7 +2352,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B18">
         <v>64.2001953125</v>
@@ -2351,7 +2384,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B22">
         <v>61.9599609375</v>
@@ -2359,7 +2392,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B23">
         <v>61.659912109375</v>
@@ -2383,7 +2416,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B26">
         <v>60.159912109375</v>
@@ -2399,7 +2432,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B28">
         <v>58.9599609375</v>
@@ -2415,79 +2448,79 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="B30">
-        <v>57.60009765625</v>
+        <v>58.25</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="1" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="B31">
-        <v>57.4599609375</v>
+        <v>57.60009765625</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="1" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="B32">
-        <v>57.449951171875</v>
+        <v>57.4599609375</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="1" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B33">
-        <v>56.9599609375</v>
+        <v>57.449951171875</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B34">
-        <v>56.260009765625</v>
+        <v>56.9599609375</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="1" t="s">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="B35">
-        <v>55.89990234375</v>
+        <v>56.260009765625</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="1" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="B36">
-        <v>54.60009765625</v>
+        <v>55.89990234375</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B37">
-        <v>54.159912109375</v>
+        <v>54.60009765625</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="1" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="B38">
-        <v>54.10009765625</v>
+        <v>54.159912109375</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
-        <v>5</v>
+        <v>47</v>
       </c>
       <c r="B39">
         <v>54.10009765625</v>
@@ -2495,55 +2528,55 @@
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="1" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B40">
-        <v>53.659912109375</v>
+        <v>54.10009765625</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="B41">
-        <v>51.56005859375</v>
+        <v>53.659912109375</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="B42">
-        <v>51.260009765625</v>
+        <v>51.56005859375</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="1" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="B43">
-        <v>49.760009765625</v>
+        <v>51.260009765625</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="1" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="B44">
-        <v>49</v>
+        <v>49.760009765625</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="1" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="B45">
-        <v>47.860107421875</v>
+        <v>49</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B46">
         <v>47.860107421875</v>
@@ -2551,57 +2584,65 @@
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B47">
-        <v>44.260009765625</v>
+        <v>47.860107421875</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="1" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="B48">
-        <v>44.06005859375</v>
+        <v>44.260009765625</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="B49">
-        <v>43.510009765625</v>
+        <v>44.06005859375</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="1" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B50">
-        <v>42.9599609375</v>
+        <v>43.510009765625</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="1" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="B51">
-        <v>40.60009765625</v>
+        <v>42.9599609375</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="B52">
-        <v>38.260009765625</v>
+        <v>40.60009765625</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B53">
+        <v>38.260009765625</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B53">
+      <c r="B54">
         <v>37.820068359375</v>
       </c>
     </row>
@@ -2612,7 +2653,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2622,7 +2663,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B2">
         <v>293.69970703125</v>
@@ -2638,7 +2679,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B4">
         <v>290.19970703125</v>
@@ -2694,7 +2735,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B11">
         <v>263.99951171875</v>
@@ -2702,7 +2743,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B12">
         <v>263.6201171875</v>
@@ -2726,7 +2767,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B15">
         <v>259.27978515625</v>
@@ -2750,7 +2791,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B18">
         <v>252.60009765625</v>
@@ -2822,7 +2863,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B27">
         <v>242.099609375</v>
@@ -2830,7 +2871,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="1" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="B28">
         <v>239.99951171875</v>
@@ -2838,7 +2879,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="B29">
         <v>239.99951171875</v>
@@ -2854,7 +2895,7 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B31">
         <v>238.1806640625</v>
@@ -2870,7 +2911,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B33">
         <v>237.330078125</v>
@@ -2878,7 +2919,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B34">
         <v>236.7998046875</v>
@@ -2950,7 +2991,7 @@
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B43">
         <v>217.81982421875</v>
@@ -2990,7 +3031,7 @@
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B48">
         <v>209.2998046875</v>
@@ -2998,7 +3039,7 @@
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B49">
         <v>206.2998046875</v>
@@ -3006,33 +3047,41 @@
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="1" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B50">
-        <v>193.91943359375</v>
+        <v>200.659912109375</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="1" t="s">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="B51">
-        <v>165.19970703125</v>
+        <v>193.91943359375</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="B52">
-        <v>145.47998046875</v>
+        <v>165.19970703125</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B53">
+        <v>145.47998046875</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B54">
         <v>145.130126953125</v>
       </c>
     </row>
@@ -3043,7 +3092,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3061,7 +3110,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -3069,7 +3118,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3077,7 +3126,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -3085,7 +3134,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -3093,7 +3142,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -3101,7 +3150,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -3109,7 +3158,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -3117,7 +3166,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -3125,7 +3174,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -3133,7 +3182,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -3141,7 +3190,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -3149,7 +3198,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -3157,7 +3206,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -3165,7 +3214,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -3173,7 +3222,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -3181,7 +3230,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -3189,7 +3238,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -3197,7 +3246,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -3205,7 +3254,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -3213,7 +3262,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -3221,7 +3270,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -3229,7 +3278,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -3237,7 +3286,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -3245,7 +3294,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -3253,7 +3302,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -3269,7 +3318,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -3277,7 +3326,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -3365,7 +3414,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -3373,7 +3422,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -3461,9 +3510,17 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="B53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54">
         <v>0</v>
       </c>
     </row>
@@ -3474,7 +3531,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3492,7 +3549,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -3500,7 +3557,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3508,7 +3565,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -3516,7 +3573,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -3524,7 +3581,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -3532,7 +3589,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -3540,7 +3597,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -3548,7 +3605,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -3556,7 +3613,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -3564,7 +3621,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -3572,7 +3629,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -3580,7 +3637,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -3588,7 +3645,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -3596,7 +3653,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -3604,7 +3661,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -3612,7 +3669,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -3620,7 +3677,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -3628,7 +3685,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -3636,7 +3693,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -3644,7 +3701,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -3652,7 +3709,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -3660,7 +3717,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -3668,7 +3725,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -3676,7 +3733,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -3684,7 +3741,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -3700,7 +3757,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -3708,7 +3765,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -3796,7 +3853,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -3804,7 +3861,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -3892,9 +3949,17 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="B53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54">
         <v>0</v>
       </c>
     </row>
@@ -3905,7 +3970,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3923,7 +3988,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -3931,7 +3996,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3939,7 +4004,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -3947,7 +4012,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -3955,7 +4020,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -3963,7 +4028,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -3971,7 +4036,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -3979,7 +4044,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -3987,7 +4052,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -3995,7 +4060,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -4003,7 +4068,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -4011,7 +4076,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -4019,7 +4084,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -4027,7 +4092,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -4035,7 +4100,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -4043,7 +4108,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -4051,7 +4116,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -4059,7 +4124,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -4067,7 +4132,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -4075,7 +4140,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -4083,7 +4148,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -4091,7 +4156,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -4099,7 +4164,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -4107,7 +4172,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -4115,7 +4180,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -4131,7 +4196,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -4139,7 +4204,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -4227,7 +4292,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -4235,7 +4300,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -4323,9 +4388,17 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="B53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54">
         <v>0</v>
       </c>
     </row>
@@ -4336,7 +4409,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -4354,7 +4427,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -4362,7 +4435,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -4370,7 +4443,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -4378,7 +4451,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -4386,7 +4459,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -4394,7 +4467,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -4402,7 +4475,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -4410,7 +4483,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -4418,7 +4491,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -4426,7 +4499,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -4434,7 +4507,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -4442,7 +4515,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -4450,7 +4523,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -4458,7 +4531,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -4466,7 +4539,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -4474,7 +4547,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -4482,7 +4555,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -4490,7 +4563,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -4498,7 +4571,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -4506,7 +4579,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -4514,7 +4587,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -4522,7 +4595,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -4530,7 +4603,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -4538,7 +4611,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -4546,7 +4619,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -4562,7 +4635,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -4570,7 +4643,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -4658,7 +4731,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -4666,7 +4739,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -4754,9 +4827,17 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="B53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona ranking de campeoes da liga classica
</commit_message>
<xml_diff>
--- a/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Completa.xlsx
+++ b/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Completa.xlsx
@@ -16,13 +16,14 @@
     <sheet name="Mes - Abril" sheetId="7" r:id="rId7"/>
     <sheet name="Mes - Maio" sheetId="8" r:id="rId8"/>
     <sheet name="Mes - Julho" sheetId="9" r:id="rId9"/>
+    <sheet name="Premiados Mensais" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="66">
   <si>
     <t>Rodada 1</t>
   </si>
@@ -202,6 +203,24 @@
   </si>
   <si>
     <t>Lider_Rodada</t>
+  </si>
+  <si>
+    <t>Mes</t>
+  </si>
+  <si>
+    <t>Posicao</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Pontos</t>
+  </si>
+  <si>
+    <t>Janeiro</t>
+  </si>
+  <si>
+    <t>Fevereiro</t>
   </si>
 </sst>
 </file>
@@ -1829,6 +1848,170 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2">
+        <v>84.85986328125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3">
+        <v>84.259765625</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4">
+        <v>74.06005859375</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5">
+        <v>73.9599609375</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6">
+        <v>73.759765625</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7">
+        <v>281.78955078125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8">
+        <v>265.3896484375</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9">
+        <v>265.3701171875</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10">
+        <v>263.08984375</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11">
+        <v>262.98974609375</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A2:A55"/>

</xml_diff>

<commit_message>
Atualiza participante da Liga Classica
</commit_message>
<xml_diff>
--- a/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Completa.xlsx
+++ b/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Completa.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="70">
   <si>
     <t>Rodada 1</t>
   </si>
@@ -94,9 +94,6 @@
     <t>FBC Colorado II</t>
   </si>
   <si>
-    <t>FC castelo Branco 2</t>
-  </si>
-  <si>
     <t>FC Los Castilho</t>
   </si>
   <si>
@@ -116,6 +113,9 @@
   </si>
   <si>
     <t>Grêmio imortal 37</t>
+  </si>
+  <si>
+    <t>HVCARTOLA</t>
   </si>
   <si>
     <t>JUV. KP</t>
@@ -206,6 +206,9 @@
   </si>
   <si>
     <t>Time do S.A.P.O</t>
+  </si>
+  <si>
+    <t>VaiDescerkkkk!!!</t>
   </si>
   <si>
     <t>VASCO MARTINS FC</t>
@@ -590,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1043,31 +1046,31 @@
         <v>22</v>
       </c>
       <c r="B15">
-        <v>37.820068359375</v>
+        <v>56.260009765625</v>
       </c>
       <c r="C15">
-        <v>64.02978515625</v>
+        <v>74.89990234375</v>
       </c>
       <c r="D15">
-        <v>78.990234375</v>
+        <v>87.33984375</v>
       </c>
       <c r="E15">
-        <v>36.580078125</v>
+        <v>69.64990234375</v>
       </c>
       <c r="F15">
-        <v>61.300048828125</v>
+        <v>88.919921875</v>
       </c>
       <c r="G15">
-        <v>68.490234375</v>
+        <v>83.419921875</v>
       </c>
       <c r="H15">
-        <v>50.8701171875</v>
+        <v>68.97021484375</v>
       </c>
       <c r="I15">
-        <v>79.35009765625</v>
+        <v>75.9501953125</v>
       </c>
       <c r="J15">
-        <v>79.35009765625</v>
+        <v>75.9501953125</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -1075,31 +1078,31 @@
         <v>23</v>
       </c>
       <c r="B16">
-        <v>56.260009765625</v>
+        <v>63.89990234375</v>
       </c>
       <c r="C16">
-        <v>74.89990234375</v>
+        <v>92.77978515625</v>
       </c>
       <c r="D16">
-        <v>87.33984375</v>
+        <v>78.39990234375</v>
       </c>
       <c r="E16">
-        <v>69.64990234375</v>
+        <v>87.64990234375</v>
       </c>
       <c r="F16">
-        <v>88.919921875</v>
+        <v>89.02001953125</v>
       </c>
       <c r="G16">
-        <v>83.419921875</v>
+        <v>62.81005859375</v>
       </c>
       <c r="H16">
-        <v>68.97021484375</v>
+        <v>105.8701171875</v>
       </c>
       <c r="I16">
-        <v>75.9501953125</v>
+        <v>76.89990234375</v>
       </c>
       <c r="J16">
-        <v>75.9501953125</v>
+        <v>76.89990234375</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -1107,31 +1110,31 @@
         <v>24</v>
       </c>
       <c r="B17">
-        <v>63.89990234375</v>
+        <v>44.06005859375</v>
       </c>
       <c r="C17">
-        <v>92.77978515625</v>
+        <v>85.7001953125</v>
       </c>
       <c r="D17">
-        <v>78.39990234375</v>
+        <v>65.259765625</v>
       </c>
       <c r="E17">
-        <v>87.64990234375</v>
+        <v>74.25</v>
       </c>
       <c r="F17">
-        <v>89.02001953125</v>
+        <v>43.39990234375</v>
       </c>
       <c r="G17">
-        <v>62.81005859375</v>
+        <v>58.68994140625</v>
       </c>
       <c r="H17">
-        <v>105.8701171875</v>
+        <v>31.6199951171875</v>
       </c>
       <c r="I17">
-        <v>76.89990234375</v>
+        <v>65.35009765625</v>
       </c>
       <c r="J17">
-        <v>76.89990234375</v>
+        <v>65.35009765625</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -1139,31 +1142,31 @@
         <v>25</v>
       </c>
       <c r="B18">
-        <v>44.06005859375</v>
+        <v>54.159912109375</v>
       </c>
       <c r="C18">
-        <v>85.7001953125</v>
+        <v>86.7001953125</v>
       </c>
       <c r="D18">
-        <v>65.259765625</v>
+        <v>75.56005859375</v>
       </c>
       <c r="E18">
-        <v>74.25</v>
+        <v>82.0498046875</v>
       </c>
       <c r="F18">
-        <v>43.39990234375</v>
+        <v>77.919921875</v>
       </c>
       <c r="G18">
-        <v>58.68994140625</v>
+        <v>73.22021484375</v>
       </c>
       <c r="H18">
-        <v>31.6199951171875</v>
+        <v>75.56982421875</v>
       </c>
       <c r="I18">
-        <v>65.35009765625</v>
+        <v>72.2998046875</v>
       </c>
       <c r="J18">
-        <v>65.35009765625</v>
+        <v>72.2998046875</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -1171,31 +1174,31 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>54.159912109375</v>
+        <v>40.60009765625</v>
       </c>
       <c r="C19">
-        <v>86.7001953125</v>
+        <v>67.8701171875</v>
       </c>
       <c r="D19">
-        <v>75.56005859375</v>
+        <v>73.64990234375</v>
       </c>
       <c r="E19">
-        <v>82.0498046875</v>
+        <v>74.02978515625</v>
       </c>
       <c r="F19">
-        <v>77.919921875</v>
+        <v>81.6201171875</v>
       </c>
       <c r="G19">
-        <v>73.22021484375</v>
+        <v>41.550048828125</v>
       </c>
       <c r="H19">
-        <v>75.56982421875</v>
+        <v>79.56982421875</v>
       </c>
       <c r="I19">
-        <v>72.2998046875</v>
+        <v>66.97998046875</v>
       </c>
       <c r="J19">
-        <v>72.2998046875</v>
+        <v>66.97998046875</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -1203,31 +1206,31 @@
         <v>27</v>
       </c>
       <c r="B20">
-        <v>40.60009765625</v>
+        <v>57.449951171875</v>
       </c>
       <c r="C20">
-        <v>67.8701171875</v>
+        <v>83.2001953125</v>
       </c>
       <c r="D20">
-        <v>73.64990234375</v>
+        <v>70.7998046875</v>
       </c>
       <c r="E20">
-        <v>74.02978515625</v>
+        <v>77.259765625</v>
       </c>
       <c r="F20">
-        <v>81.6201171875</v>
+        <v>69.3701171875</v>
       </c>
       <c r="G20">
-        <v>41.550048828125</v>
+        <v>52.199951171875</v>
       </c>
       <c r="H20">
-        <v>79.56982421875</v>
+        <v>39.969970703125</v>
       </c>
       <c r="I20">
-        <v>66.97998046875</v>
+        <v>60.5</v>
       </c>
       <c r="J20">
-        <v>66.97998046875</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -1235,31 +1238,31 @@
         <v>28</v>
       </c>
       <c r="B21">
-        <v>57.449951171875</v>
+        <v>57.60009765625</v>
       </c>
       <c r="C21">
-        <v>83.2001953125</v>
+        <v>84.5</v>
       </c>
       <c r="D21">
-        <v>70.7998046875</v>
+        <v>78.85986328125</v>
       </c>
       <c r="E21">
-        <v>77.259765625</v>
+        <v>85.97998046875</v>
       </c>
       <c r="F21">
-        <v>69.3701171875</v>
+        <v>87.22021484375</v>
       </c>
       <c r="G21">
-        <v>52.199951171875</v>
+        <v>62.10009765625</v>
       </c>
       <c r="H21">
-        <v>39.969970703125</v>
+        <v>82.81005859375</v>
       </c>
       <c r="I21">
-        <v>60.5</v>
+        <v>91.39990234375</v>
       </c>
       <c r="J21">
-        <v>60.5</v>
+        <v>91.39990234375</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -1267,31 +1270,31 @@
         <v>29</v>
       </c>
       <c r="B22">
-        <v>57.60009765625</v>
+        <v>0</v>
       </c>
       <c r="C22">
-        <v>84.5</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>78.85986328125</v>
+        <v>0</v>
       </c>
       <c r="E22">
-        <v>85.97998046875</v>
+        <v>0</v>
       </c>
       <c r="F22">
-        <v>87.22021484375</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>62.10009765625</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>82.81005859375</v>
+        <v>0</v>
       </c>
       <c r="I22">
-        <v>91.39990234375</v>
+        <v>77.18994140625</v>
       </c>
       <c r="J22">
-        <v>91.39990234375</v>
+        <v>77.18994140625</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -2259,31 +2262,31 @@
         <v>60</v>
       </c>
       <c r="B53">
-        <v>55.89990234375</v>
+        <v>44.260009765625</v>
       </c>
       <c r="C53">
-        <v>77.3798828125</v>
+        <v>90</v>
       </c>
       <c r="D53">
-        <v>43.909912109375</v>
+        <v>68.9599609375</v>
       </c>
       <c r="E53">
-        <v>76.080078125</v>
+        <v>73.22998046875</v>
       </c>
       <c r="F53">
-        <v>66.2001953125</v>
+        <v>79.33984375</v>
       </c>
       <c r="G53">
-        <v>57.780029296875</v>
+        <v>68.68994140625</v>
       </c>
       <c r="H53">
-        <v>67.33984375</v>
+        <v>61.570068359375</v>
       </c>
       <c r="I53">
-        <v>94.31982421875</v>
+        <v>74.2998046875</v>
       </c>
       <c r="J53">
-        <v>94.31982421875</v>
+        <v>74.2998046875</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -2291,30 +2294,62 @@
         <v>61</v>
       </c>
       <c r="B54">
-        <v>0</v>
+        <v>55.89990234375</v>
       </c>
       <c r="C54">
-        <v>0</v>
+        <v>77.3798828125</v>
       </c>
       <c r="D54">
-        <v>0</v>
+        <v>43.909912109375</v>
       </c>
       <c r="E54">
-        <v>0</v>
+        <v>76.080078125</v>
       </c>
       <c r="F54">
-        <v>0</v>
+        <v>66.2001953125</v>
       </c>
       <c r="G54">
-        <v>0</v>
+        <v>57.780029296875</v>
       </c>
       <c r="H54">
-        <v>0</v>
+        <v>67.33984375</v>
       </c>
       <c r="I54">
-        <v>0</v>
+        <v>94.31982421875</v>
       </c>
       <c r="J54">
+        <v>94.31982421875</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10">
+      <c r="A55" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B55">
+        <v>0</v>
+      </c>
+      <c r="C55">
+        <v>0</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>0</v>
+      </c>
+      <c r="G55">
+        <v>0</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55">
+        <v>0</v>
+      </c>
+      <c r="J55">
         <v>0</v>
       </c>
     </row>
@@ -2325,7 +2360,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2343,7 +2378,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -2351,7 +2386,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2359,7 +2394,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2367,7 +2402,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2375,7 +2410,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2383,7 +2418,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2391,7 +2426,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -2399,7 +2434,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -2407,7 +2442,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -2415,7 +2450,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -2423,7 +2458,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -2431,7 +2466,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -2439,7 +2474,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2447,7 +2482,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -2455,7 +2490,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -2463,7 +2498,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -2471,7 +2506,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -2479,7 +2514,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -2487,7 +2522,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -2495,7 +2530,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -2503,7 +2538,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -2511,7 +2546,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -2519,7 +2554,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -2527,7 +2562,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -2535,7 +2570,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -2551,7 +2586,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -2559,7 +2594,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -2647,7 +2682,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -2655,7 +2690,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -2743,9 +2778,17 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>60</v>
+        <v>33</v>
       </c>
       <c r="B53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B54">
         <v>0</v>
       </c>
     </row>
@@ -2756,7 +2799,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2774,7 +2817,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -2782,7 +2825,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2790,7 +2833,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2798,7 +2841,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2806,7 +2849,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2814,7 +2857,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2822,7 +2865,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -2830,7 +2873,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -2838,7 +2881,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -2846,7 +2889,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -2854,7 +2897,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -2862,7 +2905,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -2870,7 +2913,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2878,7 +2921,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -2886,7 +2929,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -2894,7 +2937,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -2902,7 +2945,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -2910,7 +2953,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -2918,7 +2961,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -2926,7 +2969,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -2934,7 +2977,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -2942,7 +2985,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -2950,7 +2993,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -2958,7 +3001,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -2966,7 +3009,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -2982,7 +3025,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -2990,7 +3033,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -3078,7 +3121,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -3086,7 +3129,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -3174,9 +3217,17 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>60</v>
+        <v>33</v>
       </c>
       <c r="B53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B54">
         <v>0</v>
       </c>
     </row>
@@ -3192,21 +3243,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -3220,7 +3271,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -3234,7 +3285,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -3248,7 +3299,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -3262,7 +3313,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -3276,7 +3327,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -3290,7 +3341,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8">
         <v>2</v>
@@ -3304,7 +3355,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B9">
         <v>3</v>
@@ -3318,7 +3369,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B10">
         <v>4</v>
@@ -3332,7 +3383,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B11">
         <v>5</v>
@@ -3346,7 +3397,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -3360,7 +3411,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B13">
         <v>2</v>
@@ -3374,7 +3425,7 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B14">
         <v>3</v>
@@ -3388,13 +3439,13 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B15">
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D15">
         <v>334.60009765625</v>
@@ -3402,7 +3453,7 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B16">
         <v>5</v>
@@ -3430,7 +3481,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -3883,31 +3934,31 @@
         <v>22</v>
       </c>
       <c r="B15">
-        <v>37.820068359375</v>
+        <v>56.260009765625</v>
       </c>
       <c r="C15">
-        <v>64.02978515625</v>
+        <v>74.89990234375</v>
       </c>
       <c r="D15">
-        <v>78.990234375</v>
+        <v>87.33984375</v>
       </c>
       <c r="E15">
-        <v>36.580078125</v>
+        <v>69.64990234375</v>
       </c>
       <c r="F15">
-        <v>61.300048828125</v>
+        <v>88.919921875</v>
       </c>
       <c r="G15">
-        <v>68.490234375</v>
+        <v>83.419921875</v>
       </c>
       <c r="H15">
-        <v>50.8701171875</v>
+        <v>68.97021484375</v>
       </c>
       <c r="I15">
-        <v>79.35009765625</v>
+        <v>75.9501953125</v>
       </c>
       <c r="J15">
-        <v>79.35009765625</v>
+        <v>75.9501953125</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -3915,31 +3966,31 @@
         <v>23</v>
       </c>
       <c r="B16">
-        <v>56.260009765625</v>
+        <v>63.89990234375</v>
       </c>
       <c r="C16">
-        <v>74.89990234375</v>
+        <v>92.77978515625</v>
       </c>
       <c r="D16">
-        <v>87.33984375</v>
+        <v>78.39990234375</v>
       </c>
       <c r="E16">
-        <v>69.64990234375</v>
+        <v>87.64990234375</v>
       </c>
       <c r="F16">
-        <v>88.919921875</v>
+        <v>89.02001953125</v>
       </c>
       <c r="G16">
-        <v>83.419921875</v>
+        <v>62.81005859375</v>
       </c>
       <c r="H16">
-        <v>68.97021484375</v>
+        <v>105.8701171875</v>
       </c>
       <c r="I16">
-        <v>75.9501953125</v>
+        <v>76.89990234375</v>
       </c>
       <c r="J16">
-        <v>75.9501953125</v>
+        <v>76.89990234375</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -3947,31 +3998,31 @@
         <v>24</v>
       </c>
       <c r="B17">
-        <v>63.89990234375</v>
+        <v>44.06005859375</v>
       </c>
       <c r="C17">
-        <v>92.77978515625</v>
+        <v>85.7001953125</v>
       </c>
       <c r="D17">
-        <v>78.39990234375</v>
+        <v>65.259765625</v>
       </c>
       <c r="E17">
-        <v>87.64990234375</v>
+        <v>74.25</v>
       </c>
       <c r="F17">
-        <v>89.02001953125</v>
+        <v>43.39990234375</v>
       </c>
       <c r="G17">
-        <v>62.81005859375</v>
+        <v>58.68994140625</v>
       </c>
       <c r="H17">
-        <v>105.8701171875</v>
+        <v>31.6199951171875</v>
       </c>
       <c r="I17">
-        <v>76.89990234375</v>
+        <v>65.35009765625</v>
       </c>
       <c r="J17">
-        <v>76.89990234375</v>
+        <v>65.35009765625</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -3979,31 +4030,31 @@
         <v>25</v>
       </c>
       <c r="B18">
-        <v>44.06005859375</v>
+        <v>54.159912109375</v>
       </c>
       <c r="C18">
-        <v>85.7001953125</v>
+        <v>86.7001953125</v>
       </c>
       <c r="D18">
-        <v>65.259765625</v>
+        <v>75.56005859375</v>
       </c>
       <c r="E18">
-        <v>74.25</v>
+        <v>82.0498046875</v>
       </c>
       <c r="F18">
-        <v>43.39990234375</v>
+        <v>77.919921875</v>
       </c>
       <c r="G18">
-        <v>58.68994140625</v>
+        <v>73.22021484375</v>
       </c>
       <c r="H18">
-        <v>31.6199951171875</v>
+        <v>75.56982421875</v>
       </c>
       <c r="I18">
-        <v>65.35009765625</v>
+        <v>72.2998046875</v>
       </c>
       <c r="J18">
-        <v>65.35009765625</v>
+        <v>72.2998046875</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -4011,31 +4062,31 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>54.159912109375</v>
+        <v>40.60009765625</v>
       </c>
       <c r="C19">
-        <v>86.7001953125</v>
+        <v>67.8701171875</v>
       </c>
       <c r="D19">
-        <v>75.56005859375</v>
+        <v>73.64990234375</v>
       </c>
       <c r="E19">
-        <v>82.0498046875</v>
+        <v>74.02978515625</v>
       </c>
       <c r="F19">
-        <v>77.919921875</v>
+        <v>81.6201171875</v>
       </c>
       <c r="G19">
-        <v>73.22021484375</v>
+        <v>41.550048828125</v>
       </c>
       <c r="H19">
-        <v>75.56982421875</v>
+        <v>79.56982421875</v>
       </c>
       <c r="I19">
-        <v>72.2998046875</v>
+        <v>66.97998046875</v>
       </c>
       <c r="J19">
-        <v>72.2998046875</v>
+        <v>66.97998046875</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -4043,31 +4094,31 @@
         <v>27</v>
       </c>
       <c r="B20">
-        <v>40.60009765625</v>
+        <v>57.449951171875</v>
       </c>
       <c r="C20">
-        <v>67.8701171875</v>
+        <v>83.2001953125</v>
       </c>
       <c r="D20">
-        <v>73.64990234375</v>
+        <v>70.7998046875</v>
       </c>
       <c r="E20">
-        <v>74.02978515625</v>
+        <v>77.259765625</v>
       </c>
       <c r="F20">
-        <v>81.6201171875</v>
+        <v>69.3701171875</v>
       </c>
       <c r="G20">
-        <v>41.550048828125</v>
+        <v>52.199951171875</v>
       </c>
       <c r="H20">
-        <v>79.56982421875</v>
+        <v>39.969970703125</v>
       </c>
       <c r="I20">
-        <v>66.97998046875</v>
+        <v>60.5</v>
       </c>
       <c r="J20">
-        <v>66.97998046875</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -4075,31 +4126,31 @@
         <v>28</v>
       </c>
       <c r="B21">
-        <v>57.449951171875</v>
+        <v>57.60009765625</v>
       </c>
       <c r="C21">
-        <v>83.2001953125</v>
+        <v>84.5</v>
       </c>
       <c r="D21">
-        <v>70.7998046875</v>
+        <v>78.85986328125</v>
       </c>
       <c r="E21">
-        <v>77.259765625</v>
+        <v>85.97998046875</v>
       </c>
       <c r="F21">
-        <v>69.3701171875</v>
+        <v>87.22021484375</v>
       </c>
       <c r="G21">
-        <v>52.199951171875</v>
+        <v>62.10009765625</v>
       </c>
       <c r="H21">
-        <v>39.969970703125</v>
+        <v>82.81005859375</v>
       </c>
       <c r="I21">
-        <v>60.5</v>
+        <v>91.39990234375</v>
       </c>
       <c r="J21">
-        <v>60.5</v>
+        <v>91.39990234375</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -4107,31 +4158,31 @@
         <v>29</v>
       </c>
       <c r="B22">
-        <v>57.60009765625</v>
+        <v>0</v>
       </c>
       <c r="C22">
-        <v>84.5</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>78.85986328125</v>
+        <v>0</v>
       </c>
       <c r="E22">
-        <v>85.97998046875</v>
+        <v>0</v>
       </c>
       <c r="F22">
-        <v>87.22021484375</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>62.10009765625</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>82.81005859375</v>
+        <v>0</v>
       </c>
       <c r="I22">
-        <v>91.39990234375</v>
+        <v>77.18994140625</v>
       </c>
       <c r="J22">
-        <v>91.39990234375</v>
+        <v>77.18994140625</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -5099,31 +5150,31 @@
         <v>60</v>
       </c>
       <c r="B53">
-        <v>55.89990234375</v>
+        <v>44.260009765625</v>
       </c>
       <c r="C53">
-        <v>77.3798828125</v>
+        <v>90</v>
       </c>
       <c r="D53">
-        <v>43.909912109375</v>
+        <v>68.9599609375</v>
       </c>
       <c r="E53">
-        <v>76.080078125</v>
+        <v>73.22998046875</v>
       </c>
       <c r="F53">
-        <v>66.2001953125</v>
+        <v>79.33984375</v>
       </c>
       <c r="G53">
-        <v>57.780029296875</v>
+        <v>68.68994140625</v>
       </c>
       <c r="H53">
-        <v>67.33984375</v>
+        <v>61.570068359375</v>
       </c>
       <c r="I53">
-        <v>94.31982421875</v>
+        <v>74.2998046875</v>
       </c>
       <c r="J53">
-        <v>94.31982421875</v>
+        <v>74.2998046875</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -5131,30 +5182,62 @@
         <v>61</v>
       </c>
       <c r="B54">
-        <v>0</v>
+        <v>55.89990234375</v>
       </c>
       <c r="C54">
-        <v>0</v>
+        <v>77.3798828125</v>
       </c>
       <c r="D54">
-        <v>0</v>
+        <v>43.909912109375</v>
       </c>
       <c r="E54">
-        <v>0</v>
+        <v>76.080078125</v>
       </c>
       <c r="F54">
-        <v>0</v>
+        <v>66.2001953125</v>
       </c>
       <c r="G54">
-        <v>0</v>
+        <v>57.780029296875</v>
       </c>
       <c r="H54">
-        <v>0</v>
+        <v>67.33984375</v>
       </c>
       <c r="I54">
-        <v>0</v>
+        <v>94.31982421875</v>
       </c>
       <c r="J54">
+        <v>94.31982421875</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10">
+      <c r="A55" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B55">
+        <v>0</v>
+      </c>
+      <c r="C55">
+        <v>0</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>0</v>
+      </c>
+      <c r="G55">
+        <v>0</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55">
+        <v>0</v>
+      </c>
+      <c r="J55">
         <v>0</v>
       </c>
     </row>
@@ -5165,7 +5248,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -5191,7 +5274,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4">
         <v>734.2294921875</v>
@@ -5215,7 +5298,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7">
         <v>721.8701171875</v>
@@ -5295,7 +5378,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B17">
         <v>681.360107421875</v>
@@ -5327,7 +5410,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21">
         <v>669.779541015625</v>
@@ -5450,95 +5533,95 @@
         <v>60</v>
       </c>
       <c r="B36">
-        <v>633.2294921875</v>
+        <v>634.6494140625</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="1" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="B37">
-        <v>626.02978515625</v>
+        <v>633.2294921875</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="1" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B38">
-        <v>623.7001953125</v>
+        <v>626.02978515625</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="B39">
-        <v>618.61962890625</v>
+        <v>623.7001953125</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="1" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="B40">
-        <v>617.43994140625</v>
+        <v>618.61962890625</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="B41">
-        <v>597.26953125</v>
+        <v>617.43994140625</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B42">
-        <v>594.329833984375</v>
+        <v>597.26953125</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="1" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="B43">
-        <v>592.849853515625</v>
+        <v>594.329833984375</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B44">
-        <v>571.249755859375</v>
+        <v>592.849853515625</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="B45">
-        <v>569.5693359375</v>
+        <v>571.249755859375</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="B46">
-        <v>561.649658203125</v>
+        <v>569.5693359375</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B47">
-        <v>556.78076171875</v>
+        <v>561.649658203125</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -5575,7 +5658,7 @@
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B52">
         <v>533.6800537109375</v>
@@ -5587,6 +5670,14 @@
       </c>
       <c r="B53">
         <v>462.7403564453125</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B54">
+        <v>154.3798828125</v>
       </c>
     </row>
   </sheetData>
@@ -5596,7 +5687,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:A54"/>
+  <dimension ref="A2:A55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="1:1">
@@ -5862,6 +5953,11 @@
     <row r="54" spans="1:1">
       <c r="A54" s="1" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" s="1" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -5871,7 +5967,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -5889,7 +5985,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -5897,7 +5993,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -5905,7 +6001,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -5913,7 +6009,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -5921,7 +6017,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -5929,7 +6025,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -5937,7 +6033,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -5945,7 +6041,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -5953,7 +6049,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -5961,7 +6057,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -5969,7 +6065,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -5977,7 +6073,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -5985,7 +6081,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -5993,7 +6089,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -6001,7 +6097,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -6009,7 +6105,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -6017,7 +6113,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -6025,7 +6121,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -6033,7 +6129,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -6041,7 +6137,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -6049,7 +6145,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -6057,7 +6153,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -6065,7 +6161,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -6073,7 +6169,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -6081,7 +6177,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -6097,7 +6193,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -6105,7 +6201,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -6193,7 +6289,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -6201,7 +6297,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -6289,9 +6385,17 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>60</v>
+        <v>33</v>
       </c>
       <c r="B53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B54">
         <v>0</v>
       </c>
     </row>
@@ -6302,7 +6406,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -6448,7 +6552,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B19">
         <v>63.89990234375</v>
@@ -6544,7 +6648,7 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B31">
         <v>57.60009765625</v>
@@ -6560,7 +6664,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B33">
         <v>57.449951171875</v>
@@ -6576,7 +6680,7 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B35">
         <v>56.260009765625</v>
@@ -6584,7 +6688,7 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B36">
         <v>55.89990234375</v>
@@ -6600,7 +6704,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B38">
         <v>54.159912109375</v>
@@ -6680,50 +6784,58 @@
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="1" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="B48">
-        <v>44.06005859375</v>
+        <v>44.260009765625</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="1" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="B49">
-        <v>43.510009765625</v>
+        <v>44.06005859375</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="B50">
-        <v>42.9599609375</v>
+        <v>43.510009765625</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="1" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="B51">
-        <v>40.60009765625</v>
+        <v>42.9599609375</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="1" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="B52">
-        <v>38.260009765625</v>
+        <v>40.60009765625</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B53">
-        <v>37.820068359375</v>
+        <v>38.260009765625</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B54">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6733,7 +6845,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -6791,7 +6903,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B8">
         <v>258.82958984375</v>
@@ -6815,7 +6927,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="B11">
         <v>253.08984375</v>
@@ -6823,7 +6935,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="B12">
         <v>253.08984375</v>
@@ -6839,7 +6951,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14">
         <v>249.33984375</v>
@@ -6871,7 +6983,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B18">
         <v>244.31005859375</v>
@@ -6935,210 +7047,210 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="B26">
-        <v>231.8896484375</v>
+        <v>232.18994140625</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B27">
-        <v>231.259765625</v>
+        <v>231.8896484375</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="1" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B28">
-        <v>227.90966796875</v>
+        <v>231.259765625</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B29">
-        <v>227.8095703125</v>
+        <v>227.90966796875</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="B30">
-        <v>225.2099609375</v>
+        <v>227.8095703125</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="1" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="B31">
-        <v>225.02978515625</v>
+        <v>225.2099609375</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B32">
-        <v>224.409912109375</v>
+        <v>225.02978515625</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="1" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="B33">
-        <v>222.49951171875</v>
+        <v>224.409912109375</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="1" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="B34">
-        <v>219.469482421875</v>
+        <v>222.49951171875</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B35">
-        <v>218.419921875</v>
+        <v>219.469482421875</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="1" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="B36">
-        <v>216.3896484375</v>
+        <v>218.419921875</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B37">
-        <v>216.030517578125</v>
+        <v>216.3896484375</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="1" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="B38">
-        <v>215.5498046875</v>
+        <v>216.030517578125</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B39">
-        <v>212.2099609375</v>
+        <v>215.5498046875</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B40">
-        <v>211.239990234375</v>
+        <v>212.2099609375</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="B41">
-        <v>209.509765625</v>
+        <v>211.239990234375</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B42">
-        <v>206.1201171875</v>
+        <v>209.509765625</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="1" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="B43">
-        <v>205.58984375</v>
+        <v>206.1201171875</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="1" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B44">
-        <v>204.8798828125</v>
+        <v>205.58984375</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="1" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="B45">
-        <v>199.2001953125</v>
+        <v>204.8798828125</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="1" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="B46">
-        <v>198.499755859375</v>
+        <v>199.2001953125</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="B47">
-        <v>197.369873046875</v>
+        <v>198.499755859375</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="1" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="B48">
-        <v>191.85986328125</v>
+        <v>197.369873046875</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B49">
-        <v>187.64990234375</v>
+        <v>191.85986328125</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="1" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="B50">
-        <v>186.4697265625</v>
+        <v>187.64990234375</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="1" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="B51">
-        <v>179.60009765625</v>
+        <v>186.4697265625</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -7155,6 +7267,14 @@
       </c>
       <c r="B53">
         <v>120.6300048828125</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B54">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -7164,7 +7284,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -7198,7 +7318,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B5">
         <v>334.60009765625</v>
@@ -7222,7 +7342,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B8">
         <v>323.5302734375</v>
@@ -7238,7 +7358,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B10">
         <v>317.26025390625</v>
@@ -7302,7 +7422,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B18">
         <v>299.009765625</v>
@@ -7414,7 +7534,7 @@
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B32">
         <v>285.639892578125</v>
@@ -7446,66 +7566,66 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="1" t="s">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="B36">
-        <v>282.68994140625</v>
+        <v>283.899658203125</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B37">
-        <v>280.650390625</v>
+        <v>282.68994140625</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="1" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="B38">
-        <v>279.340087890625</v>
+        <v>280.650390625</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="B39">
-        <v>277.80029296875</v>
+        <v>279.340087890625</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="1" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="B40">
-        <v>276.829833984375</v>
+        <v>277.80029296875</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="B41">
-        <v>272.47998046875</v>
+        <v>276.829833984375</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="B42">
-        <v>269.719970703125</v>
+        <v>272.47998046875</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B43">
-        <v>260.010498046875</v>
+        <v>269.719970703125</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -7558,7 +7678,7 @@
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B50">
         <v>222.0400390625</v>
@@ -7582,10 +7702,18 @@
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B53">
         <v>199.0599365234375</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B54">
+        <v>77.18994140625</v>
       </c>
     </row>
   </sheetData>
@@ -7595,7 +7723,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -7605,7 +7733,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B2">
         <v>94.31982421875</v>
@@ -7613,7 +7741,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3">
         <v>91.39990234375</v>
@@ -7709,31 +7837,31 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="B15">
-        <v>79.35009765625</v>
+        <v>79.14990234375</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>9</v>
+        <v>50</v>
       </c>
       <c r="B16">
-        <v>79.14990234375</v>
+        <v>78.0498046875</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="B17">
-        <v>78.0498046875</v>
+        <v>77.18994140625</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B18">
         <v>76.89990234375</v>
@@ -7773,7 +7901,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23">
         <v>75.9501953125</v>
@@ -7829,90 +7957,90 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="B30">
-        <v>74.0498046875</v>
+        <v>74.2998046875</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="1" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B31">
-        <v>73.4501953125</v>
+        <v>74.0498046875</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B32">
-        <v>73.35009765625</v>
+        <v>73.4501953125</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B33">
-        <v>73.14013671875</v>
+        <v>73.35009765625</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="1" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B34">
-        <v>72.2998046875</v>
+        <v>73.14013671875</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B35">
-        <v>72.25</v>
+        <v>72.2998046875</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="1" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B36">
-        <v>72.0498046875</v>
+        <v>72.25</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="1" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="B37">
-        <v>69.89990234375</v>
+        <v>72.0498046875</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B38">
-        <v>67.64990234375</v>
+        <v>69.89990234375</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B39">
-        <v>66.97998046875</v>
+        <v>67.64990234375</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="1" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="B40">
-        <v>65.60009765625</v>
+        <v>66.97998046875</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -7925,97 +8053,105 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="B42">
-        <v>65.35009765625</v>
+        <v>65.60009765625</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="1" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="B43">
-        <v>63.949951171875</v>
+        <v>65.35009765625</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="1" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B44">
-        <v>63.47998046875</v>
+        <v>63.949951171875</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B45">
-        <v>63.25</v>
+        <v>63.47998046875</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="1" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B46">
-        <v>60.5</v>
+        <v>63.25</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="B47">
-        <v>58.85009765625</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="1" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="B48">
-        <v>57.429931640625</v>
+        <v>58.85009765625</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="1" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B49">
-        <v>55.0400390625</v>
+        <v>57.429931640625</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="1" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="B50">
-        <v>54.360107421875</v>
+        <v>55.0400390625</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="1" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="B51">
-        <v>45.699951171875</v>
+        <v>54.360107421875</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B52">
-        <v>45.3701171875</v>
+        <v>45.699951171875</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B53">
+        <v>45.3701171875</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B53">
+      <c r="B54">
         <v>26.719970703125</v>
       </c>
     </row>

</xml_diff>